<commit_message>
fix: correct spelling of two student names in import data
Ufaira Afwa Khoirunnisa -> Ufairah Afwa Khoirunnisa
Kairo Malik Sopyan -> Kairo Malik Sofyan

Matches the correction already applied to the production database,
so a re-import from this sheet won't bring the old spellings back.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Asset/Data guru dan siswa kuttab Agus 2026.xlsx
+++ b/Asset/Data guru dan siswa kuttab Agus 2026.xlsx
@@ -648,7 +648,7 @@
     <t>Hawa Sigit El karimah</t>
   </si>
   <si>
-    <t>Kairo Malik Sopyan</t>
+    <t>Kairo Malik Sofyan</t>
   </si>
   <si>
     <t>M Sa'ad Salim Hadwan Saputra</t>
@@ -666,7 +666,7 @@
     <t>Sabria Hafizul Azhar</t>
   </si>
   <si>
-    <t>Ufaira Afwa Khoirunnisa</t>
+    <t>Ufairah Afwa Khoirunnisa</t>
   </si>
   <si>
     <t>Kelas</t>

</xml_diff>

<commit_message>
fix: correct class of two TK students in import data
Ufairah Afwa Khoirunnisa: Kelas TK-B2 -> Kelas TK-A
Ubaidillah Syamikh Al-Fatih: Kelas TK-A -> Kelas TK-B2

The two had their classes swapped in the sheet; this matches the
production database, which already had them in the right classes.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Asset/Data guru dan siswa kuttab Agus 2026.xlsx
+++ b/Asset/Data guru dan siswa kuttab Agus 2026.xlsx
@@ -2637,7 +2637,7 @@
         <v>187</v>
       </c>
       <c r="B147" s="1" t="s">
-        <v>41</v>
+        <v>30</v>
       </c>
     </row>
     <row r="148" spans="1:2" x14ac:dyDescent="0.25">
@@ -2805,7 +2805,7 @@
         <v>208</v>
       </c>
       <c r="B168" s="1" t="s">
-        <v>30</v>
+        <v>41</v>
       </c>
     </row>
   </sheetData>

</xml_diff>